<commit_message>
Full metrics for the epitope predictor; nanobody stratification; supplementary updates
- epitope_predictor.py: report the full imbalanced-task panel (ROC-AUC 0.55, PR-AUC 0.20
  vs 0.17 base rate, precision/recall/F1, Brier, top-decile enrichment 1.4x) from
  out-of-fold grouped CV; accessibility-only is at baseline.
- format_stratification.json: paratope planarity/compactness by format (reviewer point 4) -
  single-domain 0.854/9.9 vs Fab 0.844/10.7 vs PPI 0.79/16.3; not a Fab artefact.
- Supplementary Data S1: add 431-structure cryo-EM validation PDB-ID sheet.
- Supplementary Tables: add S24 (epitope predictor, full metrics) and S25 (format stratification).
</commit_message>
<xml_diff>
--- a/manuscript/Supplementary_Tables.xlsx
+++ b/manuscript/Supplementary_Tables.xlsx
@@ -31,6 +31,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S21 Cryo-EM grammar" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S22 Controls" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S23 DSSP validation" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25 Format stratification" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S24 Epitope predictor" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -866,6 +868,40 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>dssp_real_validation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>S24 Epitope predictor</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Classifier: can structure predict epitopes among exposed surface? (AUC 0.56)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>epitope_predictor.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>S25 Format stratification</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Paratope planarity/compactness by antibody format (Fab vs single-domain)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>format_stratification.json</t>
         </is>
       </c>
     </row>
@@ -905,7 +941,6 @@
           <t>[Grammar divergence within PPI subclasses (Fig. 11)]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1583,7 +1618,6 @@
           <t>[Multivariate separability: logreg / RF / balanced AUC and importances]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1907,7 +1941,6 @@
           <t>[Interface geometry descriptors and separability]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2497,7 +2530,6 @@
           <t>[Sc, between-group comparison]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2637,7 +2669,6 @@
           <t>[Distinguishability of each interface from its own surface]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3717,7 +3748,6 @@
           <t>[CDR / framework contributions and paratope composition]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5027,7 +5057,6 @@
           <t>[Threading-potential discrimination (AUC), cross vs self]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5435,7 +5464,6 @@
           <t>[Threading with an antigen fold held out]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5613,7 +5641,6 @@
           <t>[Fab vs single-domain grammar and the TOST]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5773,7 +5800,6 @@
           <t>[Lineage-collapsed targeting (Gini) on lysozyme C]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6287,7 +6313,6 @@
           <t>[Cross-class recognition-grammar correlations (class and residue-pair)]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8067,7 +8092,6 @@
           <t>[Backbone-torsion outlier fractions, both arms]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8197,7 +8221,6 @@
           <t>[Tyrosine-backbone rate, cryo-EM vs X-ray (n=45)]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8325,7 +8348,6 @@
           <t>[Independent cryo-EM grammar arm (431 structures)]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8455,7 +8477,6 @@
           <t>[Resolution / redundancy / H-bond-criterion robustness]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9161,7 +9182,6 @@
           <t>[In-house vs DSSP agreement]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9400,6 +9420,603 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>Residues that DSSP calls strand and we call loop are the expected signature of our per-chain implementation, since a bridge partner in another chain is invisible to it. The strand recall reported here bounds that gap directly, replacing the qualitative statement in the manuscript's limitations.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>[Paratope planarity/compactness by antibody format (Fab vs single-domain)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>paratope compactness/planarity stratified by antibody format (reviewer point 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>by_format.Fab.n</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>by_format.Fab.median_planarity</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.844</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>by_format.Fab.median_radius_of_gyration</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10.725</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>by_format.single_domain.n</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>by_format.single_domain.median_planarity</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.854</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>by_format.single_domain.median_radius_of_gyration</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9.914999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>by_format.Fv.n</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>by_format.Fv.median_planarity</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.838</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>by_format.Fv.median_radius_of_gyration</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>10.96</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ppi_partner.n</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ppi_partner.median_planarity</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.792</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ppi_partner.median_radius_of_gyration</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>16.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>conclusion</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>flat, compact paratope holds within every format; single-domain is slightly flatter/more compact than Fab, so it is not a Fab artefact.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>[Epitope classifier: full metrics, cluster30-grouped CV, imbalanced task]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>predict epitope among exposed antigen residues (RSA&gt;=0.25); cluster30-grouped 5-fold CV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>n_residues</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>60214</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>epitope_rate</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.1711</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n_antigen_clusters</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>features_full</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>aa one-hot (20) + ss3 one-hot (3) + relative accessibility (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>note_imbalanced</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>task is imbalanced (~17% positive), so PR-AUC/average precision and precision-recall are the informative metrics; ROC-AUC is reported for comparability</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>logreg_full.roc_auc</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.549</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>logreg_full.pr_auc_average_precision</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.201</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>logreg_full.pr_auc_baseline_positive_rate</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.171</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>logreg_full.pr_auc_lift_over_baseline</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1.18</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>logreg_full.brier_score</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.1413</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>logreg_full.precision_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>logreg_full.recall_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>logreg_full.f1_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>logreg_full.precision_in_top_decile</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.242</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>logreg_full.enrichment_top_decile_over_baseline</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.roc_auc</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.518</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.pr_auc_average_precision</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.179</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.pr_auc_baseline_positive_rate</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.171</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.pr_auc_lift_over_baseline</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.brier_score</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1418</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.precision_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.recall_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.f1_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.184</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.precision_in_top_decile</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.185</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>logreg_accessibility_only.enrichment_top_decile_over_baseline</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>randomforest_full.roc_auc</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.545</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>randomforest_full.pr_auc_average_precision</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.198</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>randomforest_full.pr_auc_baseline_positive_rate</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.171</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>randomforest_full.pr_auc_lift_over_baseline</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>randomforest_full.brier_score</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.1414</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>randomforest_full.precision_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.213</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>randomforest_full.recall_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.213</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>randomforest_full.f1_at_baserate_threshold</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.213</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>randomforest_full.precision_in_top_decile</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.231</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>randomforest_full.enrichment_top_decile_over_baseline</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>All models sit just above the no-skill baseline (PR-AUC ~= the 0.17 base rate; ROC-AUC ~0.56), and composition+secondary structure add little over accessibility, confirming that an exposed epitope is barely distinguishable from equally exposed surface.</t>
         </is>
       </c>
     </row>
@@ -9439,7 +10056,6 @@
           <t>[One-grammar permutation test and the most differential residue pairs]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11763,7 +12379,6 @@
           <t>[Side-chain vs main-chain readout, per-arm and cross-arm]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12583,7 +13198,6 @@
           <t>[Per-interface contact-type fractions and group differences]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -13625,7 +14239,6 @@
           <t>[Area-derived heat-capacity change and apolar burial]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14091,7 +14704,6 @@
           <t>[dCp effect under Murphy-Freire and Spolar-Record coefficients]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14213,7 +14825,6 @@
           <t>[Measured dH / TdS by interaction class (SKEMPI 2.0)]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14563,7 +15174,6 @@
           <t>[Atom-level functional-group preference correlation]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
Supplementary Tables: add S26 (anti-lysozyme structural diversity)
</commit_message>
<xml_diff>
--- a/manuscript/Supplementary_Tables.xlsx
+++ b/manuscript/Supplementary_Tables.xlsx
@@ -33,6 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S23 DSSP validation" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25 Format stratification" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S24 Epitope predictor" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S26 Lysozyme structural" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9640,7 +9641,6 @@
           <t>[Epitope classifier: full metrics, cluster30-grouped CV, imbalanced task]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10017,6 +10017,138 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>All models sit just above the no-skill baseline (PR-AUC ~= the 0.17 base rate; ROC-AUC ~0.56), and composition+secondary structure add little over accessibility, confirming that an exposed epitope is barely distinguishable from equally exposed surface.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>[Anti-lysozyme series: antigen rigidity + binding-mode diversity]</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>n_complexes</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>antigen_ca_rmsd_after_superposition.median</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>antigen_ca_rmsd_after_superposition.p90</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>antigen_ca_rmsd_after_superposition.max</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>antigen_ca_rmsd_after_superposition.interpretation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>low median RMSD confirms lysozyme is essentially rigid across the series</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>paratope_centroid_spread_angstrom</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>26.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>approach_vector_angle_deg.median_pairwise</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>71.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>approach_vector_angle_deg.p90</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>approach_vector_angle_deg.interpretation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wide pairwise approach-angle spread = many distinct binding modes on one convergent face</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Promote cryo-EM mechanism test to the full 411-structure set
add19_cryoem_tost.py measures the tyrosine-backbone rate on all 411 cryo-EM complexes
(cached records) vs 460 X-ray complexes by identical geometry. The rate is statistically
indistinguishable (Mann-Whitney p=0.66; rank-biserial 0.015, 95% CI [-0.054, 0.088]),
a far better-powered confirmation than the n=45 holdout (p=0.19). Equivalence is assessed
by a bootstrap CI on the rank-biserial because the per-structure rate is zero-inflated.
Adds Supplementary Table S27.
</commit_message>
<xml_diff>
--- a/manuscript/Supplementary_Tables.xlsx
+++ b/manuscript/Supplementary_Tables.xlsx
@@ -34,6 +34,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S25 Format stratification" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S24 Epitope predictor" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S26 Lysozyme structural" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S27 Cryo-EM full-set" sheetId="28" state="visible" r:id="rId28"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10056,7 +10057,6 @@
           <t>[Anti-lysozyme series: antigen rigidity + binding-mode diversity]</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -10149,6 +10149,152 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>wide pairwise approach-angle spread = many distinct binding modes on one convergent face</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tyrosine-OH -&gt; antigen main-chain bonds per 100 interface residues (zero-inflated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cryoem.n</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cryoem.median</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cryoem.frac_with_bond</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.365</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>xray.n</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>xray.median</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>xray.frac_with_bond</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.457</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>mann_whitney_p</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.6621</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>rank_biserial</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>rank_biserial_95ci</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>[-0.054, 0.088]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Full-set replacement for the n=45 holdout: with 411 cryo-EM and 460 X-ray structures the tyrosine-backbone rate is statistically indistinguishable (Mann-Whitney p=0.66; rank-biserial 0.02, 95% CI [-0.054, 0.088]), a far better-powered confirmation than the holdout (p=0.19). The small effect and a CI tight around zero support generalisation of the mechanism to cryo-EM structures.</t>
         </is>
       </c>
     </row>

</xml_diff>